<commit_message>
Updated knowledge base and regenerated embeddings
</commit_message>
<xml_diff>
--- a/data/knowledge_base.xlsx
+++ b/data/knowledge_base.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aditya Jaiswa\Desktop\IT_Chatbot_Project\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aditya Jaiswa\Desktop\IT_Support_Genie_AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38860B20-FD30-4CBE-88FC-6B9CB475690A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282B8647-DA9E-4C63-9426-76564E6D8733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A2B90F37-14F1-4598-89F5-58E7136E2C85}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="93">
   <si>
     <t>query</t>
   </si>
@@ -62,9 +62,6 @@
     <t>vpn error</t>
   </si>
   <si>
-    <t>cisco anyconnect not working</t>
-  </si>
-  <si>
     <t>vpn keeps disconnecting</t>
   </si>
   <si>
@@ -113,24 +110,15 @@
     <t>account locked</t>
   </si>
   <si>
-    <t>forgot password</t>
-  </si>
-  <si>
     <t>VPN</t>
   </si>
   <si>
     <t>VPN issue detected.</t>
   </si>
   <si>
-    <t>1. Restart laptop. 2. Open Cisco AnyConnect. 3. Enter VPN address. 4. Click Connect. 5. Restart AnyConnect service if fails.</t>
-  </si>
-  <si>
     <t>VPN stability issue.</t>
   </si>
   <si>
-    <t>1. Check Wi-Fi signal. 2. Disable battery saver. 3. Reinstall AnyConnect. 4. Contact IT if persists.</t>
-  </si>
-  <si>
     <t>Outlook</t>
   </si>
   <si>
@@ -143,9 +131,6 @@
     <t>Email send issue.</t>
   </si>
   <si>
-    <t>1. Check internet. 2. Check Outbox. 3. Re-enter email password. 4. Check SMTP settings.</t>
-  </si>
-  <si>
     <t>Profile issue.</t>
   </si>
   <si>
@@ -158,24 +143,15 @@
     <t>Printer offline detected.</t>
   </si>
   <si>
-    <t>1. Check printer is on. 2. Check cable. 3. Control Panel &gt; Devices and Printers. 4. Uncheck Use Printer Offline. 5. Restart Print Spooler.</t>
-  </si>
-  <si>
     <t>Printer not detected.</t>
   </si>
   <si>
-    <t>1. Restart printer. 2. Check cable. 3. Reinstall driver. 4. Add printer via Control Panel.</t>
-  </si>
-  <si>
     <t>WiFi</t>
   </si>
   <si>
     <t>Wi-Fi issue detected.</t>
   </si>
   <si>
-    <t>1. Restart laptop. 2. Forget and reconnect Wi-Fi. 3. Device Manager &gt; Update Wi-Fi driver. 4. Run Network Troubleshooter.</t>
-  </si>
-  <si>
     <t>Wi-Fi adapter issue.</t>
   </si>
   <si>
@@ -305,43 +281,125 @@
     <t>microsoft teams not loading</t>
   </si>
   <si>
-    <t>crowdstrike alert</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>SECURITY ALERT.</t>
-  </si>
-  <si>
-    <t>1. Do NOT ignore. 2. Note exact alert. 3. Do NOT open suspicious files. 4. Contact SOC immediately. 5. Give laptop hostname.</t>
-  </si>
-  <si>
-    <t>virus detected</t>
-  </si>
-  <si>
-    <t>1. Stop all work. 2. Do NOT copy files to USB. 3. Contact IT Security immediately. 4. Give laptop serial number.</t>
-  </si>
-  <si>
-    <t>malware alert</t>
-  </si>
-  <si>
-    <t>install software</t>
-  </si>
-  <si>
-    <t>Software</t>
-  </si>
-  <si>
-    <t>Software request.</t>
-  </si>
-  <si>
-    <t>1. Check Software Center first. 2. Install from there if available. 3. Raise IT ticket if not available. 4. Provide software name and business reason.</t>
-  </si>
-  <si>
-    <t>software installation</t>
-  </si>
-  <si>
-    <t>need software</t>
+    <t>1. Restart the laptop.
+2. Press the **Windows** key and open the **FortiClient VPN** application.
+3. You will see a VPN connection named **JioStar**.
+4. Click the **three-line (menu)** icon next to the connection and select **Edit Connection**.
+5. Update the VPN configuration as per the SOP.
+6. Save the changes and close the settings.
+7. Select the **JioStar** VPN connection and click **Connect**.
+8. Enter your **email ID** and **password** when prompted.
+9. If the VPN still fails to connect, restart the **FortiClient VPN** application or restart the laptop and try again.</t>
+  </si>
+  <si>
+    <t>1. Restart the laptop.
+2. Press **Windows + R**, type **`ncpa.cpl`**, and press **Enter**.
+3. Right-click the active **Wi-Fi** adapter and select **Properties**.
+4. Uncheck **Internet Protocol Version 6 (TCP/IPv6)** and click **OK**.
+5. Press the **Windows** key and open the **FortiClient VPN** application.
+6. Verify that the **JioStar** VPN connection is configured correctly as per the SOP.
+7. Click **Connect** and enter your **email ID** and **password**.
+8. Check whether the VPN connects successfully. If the issue persists, restart the **FortiClient VPN** application or restart the laptop and try again.</t>
+  </si>
+  <si>
+    <t>Forticlient Vpn not working</t>
+  </si>
+  <si>
+    <t>1. Check that the internet connection is working by opening a website in a web browser.
+2. Press the **Windows** key and open the **FortiClient VPN** application.
+3. Verify that the **JioStar** VPN configuration is correct as per the SOP.
+4. If any configuration is incorrect, update it according to the SOP and save the changes.
+5. Restart the **FortiClient VPN** application.
+6. Click **Connect** and enter your **email ID** and **password**.
+7. If the VPN still fails to connect, restart the laptop and try again.</t>
+  </si>
+  <si>
+    <t>1. Check Wi-Fi signal. 2. Disable battery saver. 3. Reinstall  Forticlient VPN app. 4. Contact IT if persists.</t>
+  </si>
+  <si>
+    <t>1. Check that the internet connection is working properly.
+2. Open **Outlook** and check the **Outbox** for any pending or stuck emails.
+3. Check the Outlook mailbox storage size.
+4. If the mailbox storage is **over 90 GB**, delete unnecessary emails and reduce the mailbox size to **at least 20 GB of free space**.
+5. Restart the laptop.
+6. Open Outlook again and verify whether the issue is resolved.</t>
+  </si>
+  <si>
+    <t>1. Open the **Personal Print Manager (PPM)** application.
+2. Check the **Jobs** tab to see if the print job is available.
+3. If the print job is not available after sending the document to print, reconfigure the **Personal Print Manager** application as per the SOP.
+4. Send the print job again and verify that it appears in the **Jobs** tab.
+5. Go to any **HP Secure Print** enabled printer.
+6. Authenticate by swiping your access card (or sign in using the configured authentication method).
+7. Verify that your print jobs are available in the **HP Secure Print** queue and release the required documents for printing.</t>
+  </si>
+  <si>
+    <t>1. Go to the **HP Secure Print** enabled printer.
+2. Log in to the printer using **`STARIN\username`** and your **Windows password**.
+3. Check whether your print jobs are available in the **HP Secure Print** queue.
+4. If the print jobs are not available, reinstall or reconfigure the **Personal Print Manager (PPM)** application as per the SOP.
+5. Send the print job again and verify that it appears in the **Jobs** tab of the **Personal Print Manager** application.
+6. Log in to the printer again and check whether the print jobs are available for release.</t>
+  </si>
+  <si>
+    <t>1. Press **Windows + R**, type **`gpedit.msc`**, and press **Enter**.
+2. Navigate to:
+   **Computer Configuration** → **Administrative Templates** → **System** → **Device Guard**.
+3. Open **Turn On Virtualization Based Security**.
+4. Select **Disabled**, then click **Apply** and **OK**.
+5. Open **Command Prompt** as **Administrator**.
+6. Run the following command:
+   ```cmd
+   gpupdate /force
+   ```
+7. Wait for the Group Policy update to complete successfully.
+8. Restart the laptop.
+9. Connect to the Wi-Fi network and verify that the issue is resolved.</t>
+  </si>
+  <si>
+    <t>1. Restart the laptop.
+2. Disconnect from the Wi-Fi network and reconnect.
+3. If the issue still persists, press **Windows + R**, type **`gpedit.msc`**, and press **Enter**.
+4. Navigate to:
+   **Computer Configuration** → **Administrative Templates** → **System** → **Device Guard**.
+5. Open **Turn On Virtualization Based Security**.
+6. Select **Disabled**, then click **Apply** and **OK**.
+7. Open **Command Prompt** as **Administrator**.
+8. Run the following command:
+   ```cmd
+   gpupdate /force
+   ```
+9. Wait for the Group Policy update to complete successfully.
+10. Restart the laptop.
+11. Connect to the Wi-Fi network and verify that the issue is resolved.</t>
+  </si>
+  <si>
+    <t>forgot email password</t>
+  </si>
+  <si>
+    <t>1. Open any web browser.
+2. Go to **[https://sspr.jiostar.com](https://sspr.jiostar.com)**.
+3. Enter your **JioStar email ID**.
+4. Complete the **CAPTCHA** verification.
+5. Click **I Forgot My Password**.
+6. Enter your **registered mobile number**.
+7. Verify your identity by entering the **OTP** sent to your mobile number.
+8. Create a new password with **at least 16 characters** that includes:
+   * One uppercase letter (A–Z)
+   * One lowercase letter (a–z)
+   * One number (0–9)
+   * One special character (e.g., `@`, `#`, `!`, `$`)
+9. Confirm the new password and submit the request.
+10. Wait for the password reset to complete, then sign in using your new password.</t>
+  </si>
+  <si>
+    <t>1. Restart the laptop.
+2. Press **Windows + R**, type **`%temp%`**, and press **Enter**. Delete all temporary files (skip any files that cannot be deleted).
+3. Press **Windows + R**, type **`temp`**, and press **Enter**. Delete all temporary files.
+4. Press **Windows + R**, type **`cleanmgr`**, and press **Enter** to open **Disk Cleanup**.
+5. Select the system drive (usually **C:**) and clean temporary files, recycle bin, and other unnecessary files.
+6. Restart the laptop again and check whether the performance has improved.
+7. If the issue persists, check for pending **Windows Updates** and install any available updates.</t>
   </si>
 </sst>
 </file>
@@ -742,13 +800,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE3F2BA-CFF2-407F-9011-1CAA936DFF08}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -765,550 +823,466 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="145" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="145" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="2" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="2" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="2" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="232" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="2" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="2" t="s">
+      <c r="D21" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="2" t="s">
+    </row>
+    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="2" t="s">
+    </row>
+    <row r="26" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="B26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="B27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+    </row>
+    <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D25" s="2" t="s">
+    </row>
+    <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D27" s="2" t="s">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+      <c r="B30" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="2" t="s">
+    </row>
+    <row r="31" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+      <c r="B31" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="2" t="s">
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D30" s="2" t="s">
+    </row>
+    <row r="33" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="B33" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="2" t="s">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>